<commit_message>
fix(#469): use in-memory terra raster read instead of grass. Should be faster. Updated tests
</commit_message>
<xml_diff>
--- a/tests/best_coverage/data/result_table.xlsx
+++ b/tests/best_coverage/data/result_table.xlsx
@@ -384,10 +384,10 @@
         <v>4</v>
       </c>
       <c r="C2">
-        <v>1863123.14356249</v>
+        <v>1863123.143562491</v>
       </c>
       <c r="D2">
-        <v>1863123.14356249</v>
+        <v>1863123.143562491</v>
       </c>
     </row>
     <row r="3">
@@ -398,10 +398,10 @@
         <v>7</v>
       </c>
       <c r="C3">
-        <v>84799.26961567999</v>
+        <v>84799.26961567998</v>
       </c>
       <c r="D3">
-        <v>1947922.41317817</v>
+        <v>1947922.413178171</v>
       </c>
     </row>
     <row r="4">
@@ -412,10 +412,10 @@
         <v>2</v>
       </c>
       <c r="C4">
-        <v>50165.9609896839</v>
+        <v>50165.96098968387</v>
       </c>
       <c r="D4">
-        <v>1998088.374167854</v>
+        <v>1998088.374167855</v>
       </c>
     </row>
     <row r="5">
@@ -426,10 +426,10 @@
         <v>6</v>
       </c>
       <c r="C5">
-        <v>14928.8159120008</v>
+        <v>14928.81591200083</v>
       </c>
       <c r="D5">
-        <v>2013017.190079855</v>
+        <v>2013017.190079856</v>
       </c>
     </row>
     <row r="6">
@@ -440,10 +440,10 @@
         <v>5</v>
       </c>
       <c r="C6">
-        <v>8129.58759221435</v>
+        <v>8129.587592214346</v>
       </c>
       <c r="D6">
-        <v>2021146.777672069</v>
+        <v>2021146.77767207</v>
       </c>
     </row>
     <row r="7">
@@ -454,10 +454,10 @@
         <v>9</v>
       </c>
       <c r="C7">
-        <v>6149.9415512085</v>
+        <v>6149.941551208496</v>
       </c>
       <c r="D7">
-        <v>2027296.719223277</v>
+        <v>2027296.719223279</v>
       </c>
     </row>
     <row r="8">
@@ -468,10 +468,10 @@
         <v>3</v>
       </c>
       <c r="C8">
-        <v>6032.97833538055</v>
+        <v>6032.978335380554</v>
       </c>
       <c r="D8">
-        <v>2033329.697558658</v>
+        <v>2033329.697558659</v>
       </c>
     </row>
     <row r="9">
@@ -482,10 +482,10 @@
         <v>8</v>
       </c>
       <c r="C9">
-        <v>3751.70513725281</v>
+        <v>3751.705137252808</v>
       </c>
       <c r="D9">
-        <v>2037081.402695911</v>
+        <v>2037081.402695912</v>
       </c>
     </row>
     <row r="10">
@@ -496,10 +496,10 @@
         <v>1</v>
       </c>
       <c r="C10">
-        <v>2513.09516716003</v>
+        <v>2513.095167160034</v>
       </c>
       <c r="D10">
-        <v>2039594.497863071</v>
+        <v>2039594.497863072</v>
       </c>
     </row>
     <row r="11">
@@ -513,7 +513,7 @@
         <v>0</v>
       </c>
       <c r="D11">
-        <v>2039594.497863071</v>
+        <v>2039594.497863072</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: restore best coverage behavior
</commit_message>
<xml_diff>
--- a/tests/best_coverage/data/result_table.xlsx
+++ b/tests/best_coverage/data/result_table.xlsx
@@ -384,10 +384,10 @@
         <v>4</v>
       </c>
       <c r="C2">
-        <v>1863123.143562491</v>
+        <v>1863123.143259477</v>
       </c>
       <c r="D2">
-        <v>1863123.143562491</v>
+        <v>1863123.143259477</v>
       </c>
     </row>
     <row r="3">
@@ -398,10 +398,10 @@
         <v>7</v>
       </c>
       <c r="C3">
-        <v>84799.26961567998</v>
+        <v>84799.26954790266</v>
       </c>
       <c r="D3">
-        <v>1947922.413178171</v>
+        <v>1947922.41280738</v>
       </c>
     </row>
     <row r="4">
@@ -412,10 +412,10 @@
         <v>2</v>
       </c>
       <c r="C4">
-        <v>50165.96098968387</v>
+        <v>50165.96088150261</v>
       </c>
       <c r="D4">
-        <v>1998088.374167855</v>
+        <v>1998088.373688883</v>
       </c>
     </row>
     <row r="5">
@@ -426,10 +426,10 @@
         <v>6</v>
       </c>
       <c r="C5">
-        <v>14928.81591200083</v>
+        <v>14928.8158991878</v>
       </c>
       <c r="D5">
-        <v>2013017.190079856</v>
+        <v>2013017.18958807</v>
       </c>
     </row>
     <row r="6">
@@ -440,10 +440,10 @@
         <v>5</v>
       </c>
       <c r="C6">
-        <v>8129.587592214346</v>
+        <v>8129.587576460402</v>
       </c>
       <c r="D6">
-        <v>2021146.77767207</v>
+        <v>2021146.777164531</v>
       </c>
     </row>
     <row r="7">
@@ -454,10 +454,10 @@
         <v>9</v>
       </c>
       <c r="C7">
-        <v>6149.941551208496</v>
+        <v>6149.941541240893</v>
       </c>
       <c r="D7">
-        <v>2027296.719223279</v>
+        <v>2027296.718705772</v>
       </c>
     </row>
     <row r="8">
@@ -468,10 +468,10 @@
         <v>3</v>
       </c>
       <c r="C8">
-        <v>6032.978335380554</v>
+        <v>6032.978334142325</v>
       </c>
       <c r="D8">
-        <v>2033329.697558659</v>
+        <v>2033329.697039914</v>
       </c>
     </row>
     <row r="9">
@@ -482,10 +482,10 @@
         <v>8</v>
       </c>
       <c r="C9">
-        <v>3751.705137252808</v>
+        <v>3751.705136057301</v>
       </c>
       <c r="D9">
-        <v>2037081.402695912</v>
+        <v>2037081.402175971</v>
       </c>
     </row>
     <row r="10">
@@ -496,10 +496,10 @@
         <v>1</v>
       </c>
       <c r="C10">
-        <v>2513.095167160034</v>
+        <v>2513.095166622566</v>
       </c>
       <c r="D10">
-        <v>2039594.497863072</v>
+        <v>2039594.497342594</v>
       </c>
     </row>
     <row r="11">
@@ -513,7 +513,7 @@
         <v>0</v>
       </c>
       <c r="D11">
-        <v>2039594.497863072</v>
+        <v>2039594.497342594</v>
       </c>
     </row>
   </sheetData>

</xml_diff>